<commit_message>
Sincronizar web y documentos con el modelo del 30-09 (cimentacion)
- IFC4X3_ADD2 re-exportado: ahora incluye las 16 zapatas (IfcFooting).
- Cifras de la seccion 08 al dia: 7 262 elementos, 56 familias, 71 categorias.
- Especificacion Tecnica: material del pilar (MT_PINO RADIATA) y paneles de
  muro cortina como "Empty" sin material.
- Tabla NDI v7 (reemplaza v6): agrega Cimentacion estructural, armazon 2X4 x16,
  material del pilar, paneles Empty, nivel/departamento de habitaciones.
- PEB completado (xlsx/pdf): mismas correcciones, nueva fila de cimentacion.
- Texto de paneles en tarjeta de materialidad y proveedores alineado al modelo.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_Documentos_Tecnicos/PEB_Pausa_Maule_completado.xlsx
+++ b/03_Documentos_Tecnicos/PEB_Pausa_Maule_completado.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/57b91da64fcc1594/Escritorio/CURSO BIM^MIA/PRACTICO/CLASE 7 SEPTIEMBRE/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\AppData\Local\Temp\claude\C--Users-user-OneDrive-Escritorio-CURSO-BIM-IA-Claude\63969694-b2af-4bd1-919d-9b63abdf2687\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_858E0603925EBA3FEC2844B64EA69E7EA47AB403" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{638F2765-FBB9-4370-BDD8-FE84BE30EA60}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8271F08F-EF8D-4164-A57E-C8E4523E4C15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4440" yWindow="4440" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1950" yWindow="1950" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BEP" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="94">
   <si>
     <t>MÉTODO TBC · THE BIM CO-WORK</t>
   </si>
@@ -145,9 +145,6 @@
     <t>NIVEL DE INFORMACIÓN (NDI) — DETALLE DEL ASPECTO 3</t>
   </si>
   <si>
-    <t>NDI 2 como base de anteproyecto, verificado en vivo contra el modelo Revit el 06-09-2026 y actualizado el 08-09-2026 tras el renombramiento de tipos/familias y la incorporacion de fichas tecnicas de Moldupanel, Arauco y Vidrios Lirquen. Tipo = informacion fija de la familia-tipo. Instancia = informacion propia de cada elemento colocado.</t>
-  </si>
-  <si>
     <t>NDI</t>
   </si>
   <si>
@@ -202,9 +199,6 @@
     <t>Paneles de muro cortina</t>
   </si>
   <si>
-    <t>PANEL_MADERA (x192). Familia de sistema System Panel. Material corregido 08-09-2026 de MT_VIDRIO (erroneo) a MT_PINO RADIATA: es un paramento solido de madera, NO vidrio. Se retiro la ficha de Vidrios Lirquen (no aplicaba).</t>
-  </si>
-  <si>
     <t>Dimension real del pano, posicion en la rejilla.</t>
   </si>
   <si>
@@ -226,9 +220,6 @@
     <t>Pilares estructurales</t>
   </si>
   <si>
-    <t>130X130 (x16). Familia: PILAR_Pino Radiata_Rectangular. Ficha Hilam MLE confirmada sin discrepancia (glulam estructural certificado NCh2148/NCh2165).</t>
-  </si>
-  <si>
     <t>Nivel base y superior, altura real, LoadBearing.</t>
   </si>
   <si>
@@ -238,9 +229,6 @@
     <t>Armazón estructural</t>
   </si>
   <si>
-    <t>2X8_PRINCIPAL (x8, 50x200mm) . 2X4_SECUNDARIA (x15, 50x100mm). Familia renombrada de 'M_Glulam-Western Species' a 'VIGA_Pino Radiata Dimensionada_Rectangular': CORRECCION 08-09-2026, no es glulam estructural sino madera dimensionada Arauco (MSD/Cepillado), material MT_PINO RADIATA. Discrepancia anterior resuelta.</t>
-  </si>
-  <si>
     <t>Longitud real, nivel, sistema de vigas al que pertenece, LoadBearing.</t>
   </si>
   <si>
@@ -277,19 +265,43 @@
     <t>No aplica: Rooms no tienen family type en Revit (TypeId = -1).</t>
   </si>
   <si>
-    <t>Nombre, Numero, Nivel, Area y Perimetro completos en las 9 habitaciones (incluye PASILLO #09, Nivel N1, 2.59 m2, agregada 08-09-2026). Departamento pendiente en las 9. Area total 79.45 m2.</t>
-  </si>
-  <si>
     <t>Analisis de programa espacial identifica con los primeros campos y contrasta el programa con los siguientes.</t>
   </si>
   <si>
-    <t>Categorías excluidas: Ventanas, muros interiores y puertas interiores no existen en el modelo. Los vanos se resuelven con seis muros cortina y la compartimentación con trece líneas de separación de habitación.</t>
-  </si>
-  <si>
     <t>Limitación conocida: los parámetros IFC de proyecto no están vinculados a las categorías de muro cortina. Exigir información alfanumérica normalizada en montantes, paneles y rejillas requiere ampliar antes esa vinculación.</t>
   </si>
   <si>
     <t>Hallazgo actualizado 08-09-2026: la familia de vigas fue renombrada de 'M_Glulam-Western Species' a 'VIGA_Pino Radiata Dimensionada_Rectangular' (resuelto). Montantes (Rectangular Mullion) y paneles (System Panel) siguen en ingles porque son familias de sistema de Revit: no se pueden renombrar (limitacion de la plataforma, no una tarea pendiente).</t>
+  </si>
+  <si>
+    <t>NDI 2 como base de anteproyecto, verificado en vivo contra el modelo Revit el 06-09-2026 y actualizado el 08-09-2026 tras el renombramiento de tipos/familias y la incorporacion de fichas tecnicas de Moldupanel, Arauco y Vidrios Lirquen. Tipo = informacion fija de la familia-tipo. Instancia = informacion propia de cada elemento colocado. Actualizado el 02-10-2026: se incorporo la categoria Cimentacion estructural (16 zapatas), se unifico el material del pilar a MT_PINO RADIATA, se corrigieron conteos (armazon 2X4 x16) y el nivel y departamento de las habitaciones.</t>
+  </si>
+  <si>
+    <t>Empty (x192). Familia de sistema System Panel (Empty System Panel). Sin material: celosia intencional, espacio libre entre los montantes de madera (decision de proyecto confirmada). Se retiro la ficha de Vidrios Lirquen (no aplicaba).</t>
+  </si>
+  <si>
+    <t>130X130 (x16). Familia: PILAR_Pino Radiata_Rectangular. Ficha Hilam MLE confirmada sin discrepancia (glulam estructural certificado NCh2148/NCh2165). Material en el modelo: MT_PINO RADIATA (unificado el 30-09-2026).</t>
+  </si>
+  <si>
+    <t>2X8_PRINCIPAL (x8, 50x200mm) . 2X4_SECUNDARIA (x16, 50x100mm). Familia renombrada de 'M_Glulam-Western Species' a 'VIGA_Pino Radiata Dimensionada_Rectangular': CORRECCION 08-09-2026, no es glulam estructural sino madera dimensionada Arauco (MSD/Cepillado), material MT_PINO RADIATA. Discrepancia anterior resuelta.</t>
+  </si>
+  <si>
+    <t>Nombre, Numero, Nivel, Area y Perimetro completos en las 9 habitaciones (incluye PASILLO #09, Nivel NPT, 2.59 m2, agregada 08-09-2026). Departamento completo en 8 de 9 (pendiente solo en PASILLO). Todas las habitaciones estan en nivel NPT. Area total 79.45 m2.</t>
+  </si>
+  <si>
+    <t>Categorías excluidas: Ventanas, muros interiores y puertas interiores no existen en el modelo. Los vanos se resuelven con seis muros cortina y la compartimentación con dieciocho líneas de separación de habitación.</t>
+  </si>
+  <si>
+    <t>Cimentación estructural</t>
+  </si>
+  <si>
+    <t>ZAPATA_Hormigon Armado_Aislada (x16, 60x60x50cm). Familia: Zapata. Material: MT_HORMIGON ARMADO (reasignado el 30-09-2026 desde el material generico de Revit). Ficha Melon (hormigon con fibra) como referencia: la resistencia 20/25/30 MPa es un rango, no un valor unico. Parametros NDI2 aun no vinculados a esta categoria.</t>
+  </si>
+  <si>
+    <t>Nivel NOG_FUNDACIONES (cota -0.20 m), posicion bajo cada pilar, Material estructural (a nivel de instancia).</t>
+  </si>
+  <si>
+    <t>Coordinacion 3D: cada zapata debe quedar bajo su pilar. Diseno de especialidades: la dimension 60x60x50 es de anteproyecto, pendiente de calculo geotecnico y estructural.</t>
   </si>
 </sst>
 </file>
@@ -532,32 +544,32 @@
     <xf numFmtId="0" fontId="13" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -795,17 +807,17 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:E39"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.54296875" customWidth="1"/>
+    <col min="1" max="1" width="11.5703125" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
     <col min="3" max="4" width="46" customWidth="1"/>
-    <col min="5" max="5" width="40.7265625" customWidth="1"/>
+    <col min="5" max="5" width="40.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="22" t="s">
+    <row r="1" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="16"/>
@@ -813,8 +825,8 @@
       <c r="D1" s="16"/>
       <c r="E1" s="1"/>
     </row>
-    <row r="2" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="25" t="s">
+    <row r="2" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="20" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="16"/>
@@ -822,8 +834,8 @@
       <c r="D2" s="16"/>
       <c r="E2" s="1"/>
     </row>
-    <row r="3" spans="1:5" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="24" t="s">
+    <row r="3" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="17" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="16"/>
@@ -831,15 +843,15 @@
       <c r="D3" s="16"/>
       <c r="E3" s="1"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
     </row>
-    <row r="5" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="15" t="s">
+    <row r="5" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="25" t="s">
         <v>3</v>
       </c>
       <c r="B5" s="16"/>
@@ -847,80 +859,80 @@
       <c r="D5" s="16"/>
       <c r="E5" s="1"/>
     </row>
-    <row r="6" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="19" t="s">
+    <row r="6" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="18"/>
-      <c r="C6" s="17" t="s">
+      <c r="B6" s="19"/>
+      <c r="C6" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="18"/>
+      <c r="D6" s="19"/>
       <c r="E6" s="1"/>
     </row>
-    <row r="7" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="19" t="s">
+    <row r="7" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="18"/>
-      <c r="C7" s="17" t="s">
+      <c r="B7" s="19"/>
+      <c r="C7" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="18"/>
+      <c r="D7" s="19"/>
       <c r="E7" s="1"/>
     </row>
-    <row r="8" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="19" t="s">
+    <row r="8" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="18"/>
-      <c r="C8" s="17" t="s">
+      <c r="B8" s="19"/>
+      <c r="C8" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="18"/>
+      <c r="D8" s="19"/>
       <c r="E8" s="1"/>
     </row>
-    <row r="9" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="19" t="s">
+    <row r="9" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="18"/>
-      <c r="C9" s="17" t="s">
+      <c r="B9" s="19"/>
+      <c r="C9" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="18"/>
+      <c r="D9" s="19"/>
       <c r="E9" s="1"/>
     </row>
-    <row r="10" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="19" t="s">
+    <row r="10" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="18"/>
-      <c r="C10" s="17" t="s">
+      <c r="B10" s="19"/>
+      <c r="C10" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="D10" s="18"/>
+      <c r="D10" s="19"/>
       <c r="E10" s="1"/>
     </row>
-    <row r="11" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="19" t="s">
+    <row r="11" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="18"/>
-      <c r="C11" s="17" t="s">
+      <c r="B11" s="19"/>
+      <c r="C11" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="D11" s="18"/>
+      <c r="D11" s="19"/>
       <c r="E11" s="1"/>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
     </row>
-    <row r="13" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>16</v>
       </c>
@@ -935,7 +947,7 @@
       </c>
       <c r="E13" s="1"/>
     </row>
-    <row r="14" spans="1:5" ht="74.150000000000006" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" ht="74.099999999999994" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>20</v>
       </c>
@@ -950,7 +962,7 @@
       </c>
       <c r="E14" s="1"/>
     </row>
-    <row r="15" spans="1:5" ht="74.150000000000006" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" ht="74.099999999999994" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>24</v>
       </c>
@@ -965,7 +977,7 @@
       </c>
       <c r="E15" s="1"/>
     </row>
-    <row r="16" spans="1:5" ht="74.150000000000006" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" ht="74.099999999999994" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>28</v>
       </c>
@@ -980,7 +992,7 @@
       </c>
       <c r="E16" s="1"/>
     </row>
-    <row r="17" spans="1:5" ht="74.150000000000006" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" ht="74.099999999999994" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>32</v>
       </c>
@@ -995,7 +1007,7 @@
       </c>
       <c r="E17" s="1"/>
     </row>
-    <row r="18" spans="1:5" ht="74.150000000000006" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" ht="74.099999999999994" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>36</v>
       </c>
@@ -1010,22 +1022,22 @@
       </c>
       <c r="E18" s="1"/>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
     </row>
-    <row r="21" spans="1:5" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="21" t="s">
+    <row r="21" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="22" t="s">
         <v>40</v>
       </c>
       <c r="B21" s="16"/>
@@ -1033,239 +1045,248 @@
       <c r="D21" s="16"/>
       <c r="E21" s="16"/>
     </row>
-    <row r="22" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="23" t="s">
-        <v>41</v>
+    <row r="22" spans="1:5" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="24" t="s">
+        <v>84</v>
       </c>
       <c r="B22" s="16"/>
       <c r="C22" s="16"/>
       <c r="D22" s="16"/>
       <c r="E22" s="16"/>
     </row>
-    <row r="24" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B24" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="B24" s="7" t="s">
+      <c r="C24" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="C24" s="7" t="s">
+      <c r="D24" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="D24" s="7" t="s">
+      <c r="E24" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="E24" s="7" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" ht="51" customHeight="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="25" spans="1:5" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="8">
         <v>2</v>
       </c>
       <c r="B25" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="C25" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="C25" s="10" t="s">
+      <c r="D25" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="D25" s="10" t="s">
+      <c r="E25" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="E25" s="10" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="26" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="11">
         <v>2</v>
       </c>
       <c r="B26" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="C26" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="C26" s="14" t="s">
+      <c r="D26" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="D26" s="13" t="s">
+      <c r="E26" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="E26" s="13" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" ht="51" customHeight="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="27" spans="1:5" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
         <v>2</v>
       </c>
       <c r="B27" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="C27" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="C27" s="13" t="s">
+      <c r="D27" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="D27" s="13" t="s">
+      <c r="E27" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="E27" s="13" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" ht="51" customHeight="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="28" spans="1:5" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A28" s="11">
         <v>2</v>
       </c>
       <c r="B28" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="C28" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="D28" s="13" t="s">
         <v>59</v>
       </c>
-      <c r="C28" s="13" t="s">
+      <c r="E28" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="D28" s="13" t="s">
-        <v>61</v>
-      </c>
-      <c r="E28" s="13" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="29" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
         <v>2</v>
       </c>
       <c r="B29" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="C29" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="D29" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="C29" s="13" t="s">
+      <c r="E29" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="D29" s="13" t="s">
-        <v>65</v>
-      </c>
-      <c r="E29" s="13" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="30" spans="1:5" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A30" s="11">
         <v>2</v>
       </c>
       <c r="B30" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="C30" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="D30" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="E30" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="C30" s="13" t="s">
-        <v>68</v>
-      </c>
-      <c r="D30" s="13" t="s">
-        <v>69</v>
-      </c>
-      <c r="E30" s="13" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" ht="51" customHeight="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="31" spans="1:5" ht="102" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
         <v>2</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C31" s="13" t="s">
-        <v>72</v>
+        <v>87</v>
       </c>
       <c r="D31" s="13" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="E31" s="13" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.35">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="102" x14ac:dyDescent="0.25">
       <c r="A32" s="11">
         <v>2</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="C32" s="13" t="s">
-        <v>76</v>
+        <v>91</v>
       </c>
       <c r="D32" s="13" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="E32" s="13" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.35">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="11">
         <v>2</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="C33" s="13" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="D33" s="13" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="E33" s="13" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.35">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="11">
         <v>2</v>
       </c>
       <c r="B34" s="12" t="s">
-        <v>83</v>
-      </c>
-      <c r="C34" s="14" t="s">
-        <v>84</v>
+        <v>75</v>
+      </c>
+      <c r="C34" s="13" t="s">
+        <v>76</v>
       </c>
       <c r="D34" s="13" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="E34" s="13" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" ht="26.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="20" t="s">
-        <v>87</v>
-      </c>
-      <c r="B36" s="16"/>
-      <c r="C36" s="16"/>
-      <c r="D36" s="16"/>
-      <c r="E36" s="16"/>
-    </row>
-    <row r="37" spans="1:5" ht="26.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="20" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="76.5" x14ac:dyDescent="0.25">
+      <c r="A35" s="11">
+        <v>2</v>
+      </c>
+      <c r="B35" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="C35" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="D35" s="13" t="s">
         <v>88</v>
+      </c>
+      <c r="E35" s="13" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="15" t="s">
+        <v>89</v>
       </c>
       <c r="B37" s="16"/>
       <c r="C37" s="16"/>
       <c r="D37" s="16"/>
       <c r="E37" s="16"/>
     </row>
-    <row r="38" spans="1:5" ht="26.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="20" t="s">
-        <v>89</v>
+    <row r="38" spans="1:5" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="15" t="s">
+        <v>82</v>
       </c>
       <c r="B38" s="16"/>
       <c r="C38" s="16"/>
       <c r="D38" s="16"/>
       <c r="E38" s="16"/>
     </row>
+    <row r="39" spans="1:5" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="15" t="s">
+        <v>83</v>
+      </c>
+      <c r="B39" s="16"/>
+      <c r="C39" s="16"/>
+      <c r="D39" s="16"/>
+      <c r="E39" s="16"/>
+    </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="A38:E38"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A37:E37"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="A21:E21"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="A8:B8"/>
@@ -1275,10 +1296,18 @@
     <mergeCell ref="A5:D5"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A36:E36"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A39:E39"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A38:E38"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="A21:E21"/>
+    <mergeCell ref="A37:E37"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="36" orientation="landscape" r:id="rId1"/>

</xml_diff>

<commit_message>
Actualizar lamina, isometricas, parametros NDI2 y paquete de descarga
- Lamina A101 (pdf/jpg) e isometricas re-exportadas desde Revit: ahora
  muestran las 16 zapatas y el nivel de fundaciones.
- Parametros compartidos NDI2 vinculados a Cimentacion estructural en el
  modelo; listado de parametros v3 (reemplaza al v2) y Tabla NDI v7 al dia.
- PEB completado y Fichas de proveedores alineados con el modelo (paneles
  Empty, zapatas con ficha Melon).
- Paquete de descarga: .rar desactualizado reemplazado por .zip con los
  documentos vigentes; tarjeta de hormigon y tabla de proveedores mencionan
  las zapatas.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_Documentos_Tecnicos/PEB_Pausa_Maule_completado.xlsx
+++ b/03_Documentos_Tecnicos/PEB_Pausa_Maule_completado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\AppData\Local\Temp\claude\C--Users-user-OneDrive-Escritorio-CURSO-BIM-IA-Claude\63969694-b2af-4bd1-919d-9b63abdf2687\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8271F08F-EF8D-4164-A57E-C8E4523E4C15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA605CF3-0398-4CB8-9AEF-1FD7375BB5CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1950" yWindow="1950" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -274,9 +274,6 @@
     <t>Hallazgo actualizado 08-09-2026: la familia de vigas fue renombrada de 'M_Glulam-Western Species' a 'VIGA_Pino Radiata Dimensionada_Rectangular' (resuelto). Montantes (Rectangular Mullion) y paneles (System Panel) siguen en ingles porque son familias de sistema de Revit: no se pueden renombrar (limitacion de la plataforma, no una tarea pendiente).</t>
   </si>
   <si>
-    <t>NDI 2 como base de anteproyecto, verificado en vivo contra el modelo Revit el 06-09-2026 y actualizado el 08-09-2026 tras el renombramiento de tipos/familias y la incorporacion de fichas tecnicas de Moldupanel, Arauco y Vidrios Lirquen. Tipo = informacion fija de la familia-tipo. Instancia = informacion propia de cada elemento colocado. Actualizado el 02-10-2026: se incorporo la categoria Cimentacion estructural (16 zapatas), se unifico el material del pilar a MT_PINO RADIATA, se corrigieron conteos (armazon 2X4 x16) y el nivel y departamento de las habitaciones.</t>
-  </si>
-  <si>
     <t>Empty (x192). Familia de sistema System Panel (Empty System Panel). Sin material: celosia intencional, espacio libre entre los montantes de madera (decision de proyecto confirmada). Se retiro la ficha de Vidrios Lirquen (no aplicaba).</t>
   </si>
   <si>
@@ -295,13 +292,16 @@
     <t>Cimentación estructural</t>
   </si>
   <si>
-    <t>ZAPATA_Hormigon Armado_Aislada (x16, 60x60x50cm). Familia: Zapata. Material: MT_HORMIGON ARMADO (reasignado el 30-09-2026 desde el material generico de Revit). Ficha Melon (hormigon con fibra) como referencia: la resistencia 20/25/30 MPa es un rango, no un valor unico. Parametros NDI2 aun no vinculados a esta categoria.</t>
-  </si>
-  <si>
     <t>Nivel NOG_FUNDACIONES (cota -0.20 m), posicion bajo cada pilar, Material estructural (a nivel de instancia).</t>
   </si>
   <si>
     <t>Coordinacion 3D: cada zapata debe quedar bajo su pilar. Diseno de especialidades: la dimension 60x60x50 es de anteproyecto, pendiente de calculo geotecnico y estructural.</t>
+  </si>
+  <si>
+    <t>ZAPATA_Hormigon Armado_Aislada (x16, 60x60x50cm). Familia: Zapata. Material: MT_HORMIGON ARMADO (reasignado el 30-09-2026 desde el material generico de Revit). Ficha Melon (hormigon con fibra) como referencia: la resistencia 20/25/30 MPa es un rango, no un valor unico. NDI2_Fuente_Ficha y NDI2_Observacion vinculados a esta categoria y con valores (02-10-2026).</t>
+  </si>
+  <si>
+    <t>NDI 2 como base de anteproyecto, verificado en vivo contra el modelo Revit el 06-09-2026 y actualizado el 08-09-2026 tras el renombramiento de tipos/familias y la incorporacion de fichas tecnicas de Moldupanel, Arauco y Vidrios Lirquen. Tipo = informacion fija de la familia-tipo. Instancia = informacion propia de cada elemento colocado. Actualizado el 02-10-2026: se incorporo la categoria Cimentacion estructural (16 zapatas, con parametros NDI2 vinculados), se unifico el material del pilar a MT_PINO RADIATA, se corrigieron conteos (armazon 2X4 x16) y el nivel y departamento de las habitaciones.</t>
   </si>
 </sst>
 </file>
@@ -544,31 +544,31 @@
     <xf numFmtId="0" fontId="13" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -817,7 +817,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="16"/>
@@ -826,7 +826,7 @@
       <c r="E1" s="1"/>
     </row>
     <row r="2" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="24" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="16"/>
@@ -835,7 +835,7 @@
       <c r="E2" s="1"/>
     </row>
     <row r="3" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="17" t="s">
+      <c r="A3" s="23" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="16"/>
@@ -851,7 +851,7 @@
       <c r="E4" s="1"/>
     </row>
     <row r="5" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="25" t="s">
+      <c r="A5" s="21" t="s">
         <v>3</v>
       </c>
       <c r="B5" s="16"/>
@@ -860,69 +860,69 @@
       <c r="E5" s="1"/>
     </row>
     <row r="6" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="19"/>
-      <c r="C6" s="21" t="s">
+      <c r="B6" s="18"/>
+      <c r="C6" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="19"/>
+      <c r="D6" s="18"/>
       <c r="E6" s="1"/>
     </row>
     <row r="7" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="18" t="s">
+      <c r="A7" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="19"/>
-      <c r="C7" s="21" t="s">
+      <c r="B7" s="18"/>
+      <c r="C7" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="19"/>
+      <c r="D7" s="18"/>
       <c r="E7" s="1"/>
     </row>
     <row r="8" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="18" t="s">
+      <c r="A8" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="19"/>
-      <c r="C8" s="21" t="s">
+      <c r="B8" s="18"/>
+      <c r="C8" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="19"/>
+      <c r="D8" s="18"/>
       <c r="E8" s="1"/>
     </row>
     <row r="9" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="18" t="s">
+      <c r="A9" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="19"/>
-      <c r="C9" s="21" t="s">
+      <c r="B9" s="18"/>
+      <c r="C9" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="19"/>
+      <c r="D9" s="18"/>
       <c r="E9" s="1"/>
     </row>
     <row r="10" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="19"/>
-      <c r="C10" s="21" t="s">
+      <c r="B10" s="18"/>
+      <c r="C10" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="D10" s="19"/>
+      <c r="D10" s="18"/>
       <c r="E10" s="1"/>
     </row>
     <row r="11" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="18" t="s">
+      <c r="A11" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="19"/>
-      <c r="C11" s="21" t="s">
+      <c r="B11" s="18"/>
+      <c r="C11" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="D11" s="19"/>
+      <c r="D11" s="18"/>
       <c r="E11" s="1"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -1037,7 +1037,7 @@
       <c r="E20" s="1"/>
     </row>
     <row r="21" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="22" t="s">
+      <c r="A21" s="25" t="s">
         <v>40</v>
       </c>
       <c r="B21" s="16"/>
@@ -1046,8 +1046,8 @@
       <c r="E21" s="16"/>
     </row>
     <row r="22" spans="1:5" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="24" t="s">
-        <v>84</v>
+      <c r="A22" s="20" t="s">
+        <v>93</v>
       </c>
       <c r="B22" s="16"/>
       <c r="C22" s="16"/>
@@ -1130,7 +1130,7 @@
         <v>58</v>
       </c>
       <c r="C28" s="13" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D28" s="13" t="s">
         <v>59</v>
@@ -1164,7 +1164,7 @@
         <v>65</v>
       </c>
       <c r="C30" s="13" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D30" s="13" t="s">
         <v>66</v>
@@ -1181,7 +1181,7 @@
         <v>68</v>
       </c>
       <c r="C31" s="13" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D31" s="13" t="s">
         <v>69</v>
@@ -1190,21 +1190,21 @@
         <v>70</v>
       </c>
     </row>
-    <row r="32" spans="1:5" ht="102" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" ht="114.75" x14ac:dyDescent="0.25">
       <c r="A32" s="11">
         <v>2</v>
       </c>
       <c r="B32" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="C32" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="D32" s="13" t="s">
         <v>90</v>
       </c>
-      <c r="C32" s="13" t="s">
+      <c r="E32" s="13" t="s">
         <v>91</v>
-      </c>
-      <c r="D32" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="E32" s="13" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1252,15 +1252,15 @@
         <v>80</v>
       </c>
       <c r="D35" s="13" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E35" s="13" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="15" t="s">
-        <v>89</v>
+      <c r="A37" s="22" t="s">
+        <v>88</v>
       </c>
       <c r="B37" s="16"/>
       <c r="C37" s="16"/>
@@ -1268,7 +1268,7 @@
       <c r="E37" s="16"/>
     </row>
     <row r="38" spans="1:5" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="15" t="s">
+      <c r="A38" s="22" t="s">
         <v>82</v>
       </c>
       <c r="B38" s="16"/>
@@ -1277,7 +1277,7 @@
       <c r="E38" s="16"/>
     </row>
     <row r="39" spans="1:5" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="15" t="s">
+      <c r="A39" s="22" t="s">
         <v>83</v>
       </c>
       <c r="B39" s="16"/>
@@ -1287,6 +1287,15 @@
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="A39:E39"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A38:E38"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="A21:E21"/>
+    <mergeCell ref="A37:E37"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="A8:B8"/>
@@ -1299,15 +1308,6 @@
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A39:E39"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A38:E38"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="A21:E21"/>
-    <mergeCell ref="A37:E37"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="36" orientation="landscape" r:id="rId1"/>

</xml_diff>

<commit_message>
Cantidades del modelo, NDI v8, Parámetros v4, PEB actualizado (IsExternal y LoadBearing resueltos), .rvt actualizado, respaldo si no se activan las animaciones
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_Documentos_Tecnicos/PEB_Pausa_Maule_completado.xlsx
+++ b/03_Documentos_Tecnicos/PEB_Pausa_Maule_completado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\AppData\Local\Temp\claude\C--Users-user-OneDrive-Escritorio-CURSO-BIM-IA-Claude\63969694-b2af-4bd1-919d-9b63abdf2687\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA605CF3-0398-4CB8-9AEF-1FD7375BB5CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{612709D2-8710-4067-9FDA-FA69BC2125FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1950" yWindow="1950" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -166,12 +166,6 @@
     <t>MURO_EXT_QUINCHA_12cm (x11) . MURO_CORTINA_EXT_MADERA (x6). Familias: Muro basico / Muro cortina. Nivel tipo: espesor de capas y material (material real: MT_TIERRA_QUINCHA; ficha CONSTRUCCION_CON_QUINCHA_LIVIANA_1a_edicion.pdf).</t>
   </si>
   <si>
-    <t>Nivel base y superior, longitud real del tramo. IsExternal y LoadBearing viven en instancia (ambos vacios hoy).</t>
-  </si>
-  <si>
-    <t>Coordinacion 3D necesita espesor y posicion reales para el encuentro con pilares y cubierta. Diseno de especialidades usa LoadBearing para separar quincha portante de muro cortina.</t>
-  </si>
-  <si>
     <t>Rejillas de muro cortina</t>
   </si>
   <si>
@@ -220,18 +214,12 @@
     <t>Pilares estructurales</t>
   </si>
   <si>
-    <t>Nivel base y superior, altura real, LoadBearing.</t>
-  </si>
-  <si>
     <t>Coordinacion 3D: el pilar choca con muros y vigas. La seccion debe ser dato del tipo, no solo su nombre.</t>
   </si>
   <si>
     <t>Armazón estructural</t>
   </si>
   <si>
-    <t>Longitud real, nivel, sistema de vigas al que pertenece, LoadBearing.</t>
-  </si>
-  <si>
     <t>Revision del diseno comprueba la jerarquia entre principales y secundarias, ya resuelta en los tipos.</t>
   </si>
   <si>
@@ -302,6 +290,18 @@
   </si>
   <si>
     <t>NDI 2 como base de anteproyecto, verificado en vivo contra el modelo Revit el 06-09-2026 y actualizado el 08-09-2026 tras el renombramiento de tipos/familias y la incorporacion de fichas tecnicas de Moldupanel, Arauco y Vidrios Lirquen. Tipo = informacion fija de la familia-tipo. Instancia = informacion propia de cada elemento colocado. Actualizado el 02-10-2026: se incorporo la categoria Cimentacion estructural (16 zapatas, con parametros NDI2 vinculados), se unifico el material del pilar a MT_PINO RADIATA, se corrigieron conteos (armazon 2X4 x16) y el nivel y departamento de las habitaciones.</t>
+  </si>
+  <si>
+    <t>Nivel base y superior, longitud real del tramo. IsExternal = Si en los 17 muros (tipo e instancia, 02-10-2026); LoadBearing no esta vinculado a esta categoria.</t>
+  </si>
+  <si>
+    <t>Coordinacion 3D necesita espesor y posicion reales para el encuentro con pilares y cubierta. Diseno de especialidades usa IsExternal para separar muros de fachada de la compartimentacion.</t>
+  </si>
+  <si>
+    <t>Nivel base y superior, altura real. LoadBearing (de tipo) = 1.</t>
+  </si>
+  <si>
+    <t>Longitud real, nivel, sistema de vigas al que pertenece. LoadBearing (de tipo) = 1.</t>
   </si>
 </sst>
 </file>
@@ -544,31 +544,31 @@
     <xf numFmtId="0" fontId="13" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -817,7 +817,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="16"/>
@@ -826,7 +826,7 @@
       <c r="E1" s="1"/>
     </row>
     <row r="2" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="20" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="16"/>
@@ -835,7 +835,7 @@
       <c r="E2" s="1"/>
     </row>
     <row r="3" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="23" t="s">
+      <c r="A3" s="17" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="16"/>
@@ -851,7 +851,7 @@
       <c r="E4" s="1"/>
     </row>
     <row r="5" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="21" t="s">
+      <c r="A5" s="25" t="s">
         <v>3</v>
       </c>
       <c r="B5" s="16"/>
@@ -860,69 +860,69 @@
       <c r="E5" s="1"/>
     </row>
     <row r="6" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="18"/>
-      <c r="C6" s="17" t="s">
+      <c r="B6" s="19"/>
+      <c r="C6" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="18"/>
+      <c r="D6" s="19"/>
       <c r="E6" s="1"/>
     </row>
     <row r="7" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="18"/>
-      <c r="C7" s="17" t="s">
+      <c r="B7" s="19"/>
+      <c r="C7" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="18"/>
+      <c r="D7" s="19"/>
       <c r="E7" s="1"/>
     </row>
     <row r="8" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="19" t="s">
+      <c r="A8" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="18"/>
-      <c r="C8" s="17" t="s">
+      <c r="B8" s="19"/>
+      <c r="C8" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="18"/>
+      <c r="D8" s="19"/>
       <c r="E8" s="1"/>
     </row>
     <row r="9" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="18"/>
-      <c r="C9" s="17" t="s">
+      <c r="B9" s="19"/>
+      <c r="C9" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="18"/>
+      <c r="D9" s="19"/>
       <c r="E9" s="1"/>
     </row>
     <row r="10" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="19" t="s">
+      <c r="A10" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="18"/>
-      <c r="C10" s="17" t="s">
+      <c r="B10" s="19"/>
+      <c r="C10" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="D10" s="18"/>
+      <c r="D10" s="19"/>
       <c r="E10" s="1"/>
     </row>
     <row r="11" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="18"/>
-      <c r="C11" s="17" t="s">
+      <c r="B11" s="19"/>
+      <c r="C11" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="D11" s="18"/>
+      <c r="D11" s="19"/>
       <c r="E11" s="1"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -1037,7 +1037,7 @@
       <c r="E20" s="1"/>
     </row>
     <row r="21" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="25" t="s">
+      <c r="A21" s="22" t="s">
         <v>40</v>
       </c>
       <c r="B21" s="16"/>
@@ -1046,8 +1046,8 @@
       <c r="E21" s="16"/>
     </row>
     <row r="22" spans="1:5" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="20" t="s">
-        <v>93</v>
+      <c r="A22" s="24" t="s">
+        <v>89</v>
       </c>
       <c r="B22" s="16"/>
       <c r="C22" s="16"/>
@@ -1071,7 +1071,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="25" spans="1:5" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A25" s="8">
         <v>2</v>
       </c>
@@ -1082,10 +1082,10 @@
         <v>47</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>48</v>
+        <v>90</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>49</v>
+        <v>91</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1093,16 +1093,16 @@
         <v>2</v>
       </c>
       <c r="B26" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="C26" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="D26" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="C26" s="14" t="s">
+      <c r="E26" s="13" t="s">
         <v>51</v>
-      </c>
-      <c r="D26" s="13" t="s">
-        <v>52</v>
-      </c>
-      <c r="E26" s="13" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="51" customHeight="1" x14ac:dyDescent="0.25">
@@ -1110,16 +1110,16 @@
         <v>2</v>
       </c>
       <c r="B27" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="C27" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="D27" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="C27" s="13" t="s">
+      <c r="E27" s="13" t="s">
         <v>55</v>
-      </c>
-      <c r="D27" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="E27" s="13" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="63.75" x14ac:dyDescent="0.25">
@@ -1127,16 +1127,16 @@
         <v>2</v>
       </c>
       <c r="B28" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="C28" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="D28" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="E28" s="13" t="s">
         <v>58</v>
-      </c>
-      <c r="C28" s="13" t="s">
-        <v>84</v>
-      </c>
-      <c r="D28" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="E28" s="13" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1144,16 +1144,16 @@
         <v>2</v>
       </c>
       <c r="B29" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="C29" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="D29" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="C29" s="13" t="s">
+      <c r="E29" s="13" t="s">
         <v>62</v>
-      </c>
-      <c r="D29" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="E29" s="13" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="63.75" x14ac:dyDescent="0.25">
@@ -1161,16 +1161,16 @@
         <v>2</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C30" s="13" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="D30" s="13" t="s">
-        <v>66</v>
+        <v>92</v>
       </c>
       <c r="E30" s="13" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="102" x14ac:dyDescent="0.25">
@@ -1178,16 +1178,16 @@
         <v>2</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C31" s="13" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="D31" s="13" t="s">
-        <v>69</v>
+        <v>93</v>
       </c>
       <c r="E31" s="13" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="114.75" x14ac:dyDescent="0.25">
@@ -1195,16 +1195,16 @@
         <v>2</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C32" s="13" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="D32" s="13" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="E32" s="13" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1212,16 +1212,16 @@
         <v>2</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C33" s="13" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="D33" s="13" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="E33" s="13" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1229,16 +1229,16 @@
         <v>2</v>
       </c>
       <c r="B34" s="12" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C34" s="13" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="D34" s="13" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="E34" s="13" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="76.5" x14ac:dyDescent="0.25">
@@ -1246,21 +1246,21 @@
         <v>2</v>
       </c>
       <c r="B35" s="12" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="C35" s="14" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="D35" s="13" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="E35" s="13" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="22" t="s">
-        <v>88</v>
+      <c r="A37" s="15" t="s">
+        <v>84</v>
       </c>
       <c r="B37" s="16"/>
       <c r="C37" s="16"/>
@@ -1268,8 +1268,8 @@
       <c r="E37" s="16"/>
     </row>
     <row r="38" spans="1:5" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="22" t="s">
-        <v>82</v>
+      <c r="A38" s="15" t="s">
+        <v>78</v>
       </c>
       <c r="B38" s="16"/>
       <c r="C38" s="16"/>
@@ -1277,8 +1277,8 @@
       <c r="E38" s="16"/>
     </row>
     <row r="39" spans="1:5" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="22" t="s">
-        <v>83</v>
+      <c r="A39" s="15" t="s">
+        <v>79</v>
       </c>
       <c r="B39" s="16"/>
       <c r="C39" s="16"/>
@@ -1287,15 +1287,6 @@
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="A39:E39"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A38:E38"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="A21:E21"/>
-    <mergeCell ref="A37:E37"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="A8:B8"/>
@@ -1308,6 +1299,15 @@
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A39:E39"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A38:E38"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="A21:E21"/>
+    <mergeCell ref="A37:E37"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="36" orientation="landscape" r:id="rId1"/>

</xml_diff>